<commit_message>
Off-prem MPO: refresh September data through 9/11, merge Promos_Report_13
Four RDE exports plus the promos report onto the cooler-door archive.
Constellation 598 -> 726 placements (Shane Barreca newly at goal),
Keystone 101 -> 109 buying accounts (still 3 reps at 40%), Fever Tree
39 -> 60 new placements, Wine & Spirits 122 -> 147 (9 -> 13 reps at
goal), POS cooler doors 12 -> 20 stickers (Derrick Laws joins Chris
Payton at goal). No rep lost ground; the seven Wine & Spirits rows that
left the export were re-dated or reassigned, not dropped.

Keystone moved with keystone-ice (actuals.csv on the same 124-row
export, 109 accounts on both) and incentive-tracking was rebuilt after
it, per the shared-export sync rule.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012WazBFfRJ9rk1xXi61Nw4p
</commit_message>
<xml_diff>
--- a/MPOs/off-prem/pos_cooler_door_promos.xlsx
+++ b/MPOs/off-prem/pos_cooler_door_promos.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.7109375" customWidth="1" style="6" min="1" max="1"/>
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:34 AM</t>
+          <t>09/09/2026 10:37 AM</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -629,22 +629,22 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>WINELAND</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>50020</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>247 DEGRAW AVE</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>TEANECK</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -659,14 +659,10 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>CARBLISS</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>DRINK CARBLISS</t>
-        </is>
-      </c>
+          <t>MONACO</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="n"/>
       <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -676,7 +672,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:33 AM</t>
+          <t>09/08/2026 12:28 PM</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -686,12 +682,12 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -714,22 +710,22 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -744,7 +740,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>TRULY HARD SELTZER</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -761,7 +757,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:32 AM</t>
+          <t>09/08/2026 12:28 PM</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -771,12 +767,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -799,22 +795,22 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -829,7 +825,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>BLUE MOON BELGIAN WHITE ALE</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -846,7 +842,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:31 AM</t>
+          <t>09/08/2026 12:17 PM</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -856,12 +852,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -884,22 +880,22 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>RAPHAEL &amp; ANGEL LIQ (A)</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>20080</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>390 MAIN ST</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -914,12 +910,12 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
@@ -931,22 +927,22 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:31 AM</t>
+          <t>09/08/2026 11:37 AM</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -969,22 +965,22 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -999,7 +995,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>MODELO CHELADA</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1016,22 +1012,22 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:30 AM</t>
+          <t>09/08/2026 11:35 AM</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1054,22 +1050,22 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -1084,12 +1080,12 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>CERVEZA REPUBLICA LA TUYA 5.0 LA DURA</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>VINAIO IMPORTS LTD</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
@@ -1101,22 +1097,22 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:29 AM</t>
+          <t>09/08/2026 11:34 AM</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1139,22 +1135,22 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1169,12 +1165,12 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>MODELO ORO</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
@@ -1186,22 +1182,22 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:11 AM</t>
+          <t>09/08/2026 11:32 AM</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1224,22 +1220,22 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>FAIR LAWN WINE &amp; SPIRITS</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>81006</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>21-00 MAPLE AVE</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>FAIR LAWN</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -1254,12 +1250,12 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
@@ -1271,12 +1267,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:31 AM</t>
+          <t>09/03/2026 11:34 AM</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1309,22 +1305,22 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1356,12 +1352,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:30 AM</t>
+          <t>09/03/2026 11:33 AM</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1394,22 +1390,22 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -1424,12 +1420,12 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>TRULY HARD SELTZER</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q11" s="3" t="inlineStr">
@@ -1441,12 +1437,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:29 AM</t>
+          <t>09/03/2026 11:32 AM</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1479,22 +1475,22 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -1509,12 +1505,12 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q12" s="3" t="inlineStr">
@@ -1526,12 +1522,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:28 AM</t>
+          <t>09/03/2026 11:31 AM</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1564,22 +1560,22 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1594,12 +1590,12 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr">
@@ -1611,12 +1607,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:28 AM</t>
+          <t>09/03/2026 11:31 AM</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1649,22 +1645,22 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -1679,12 +1675,12 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>MILLER LITE BEER</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q14" s="3" t="inlineStr">
@@ -1696,83 +1692,763 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>09/03/2026 11:30 AM</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>76010</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>66 MARKET ST</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>SADDLE BROOK</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>CAPE MAY BREWING COMPANY</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>CAPE MAY BREWING COMPANY</t>
+        </is>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 11:29 AM</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>76010</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>66 MARKET ST</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>SADDLE BROOK</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>SUN CRUISERS RTD</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>BOSTON BEER COMPANY</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 11:11 AM</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Mike Ast</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>FAIR LAWN WINE &amp; SPIRITS</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>81006</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>21-00 MAPLE AVE</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>FAIR LAWN</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>SUN CRUISERS RTD</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>BOSTON BEER COMPANY</t>
+        </is>
+      </c>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:31 AM</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>CARBLISS</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>DRINK CARBLISS</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:30 AM</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>CORONA EXTRA</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>CONSTELLATION BRANDS</t>
+        </is>
+      </c>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:29 AM</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>MODELO ESPECIAL</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>CONSTELLATION BRANDS</t>
+        </is>
+      </c>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:28 AM</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>11.1</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>COORS LIGHT BEER</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
+        </is>
+      </c>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:28 AM</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>MILLER LITE BEER</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>09/03/2026 10:27 AM</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>12.1</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Chris Payton</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Michael Engel</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>Ashley Furman</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Sales Rep</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>Feature Activation</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="H23" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>CLIFTON DISC LIQ (A)</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>25045</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>73 ACKERMAN AVE BOTONY PL</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>CLIFTON</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M23" s="2" t="inlineStr">
         <is>
           <t>MBO</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N23" s="2" t="inlineStr">
         <is>
           <t>Cooler Door Wrap</t>
         </is>
       </c>
-      <c r="O15" s="2" t="inlineStr">
+      <c r="O23" s="2" t="inlineStr">
         <is>
           <t>MODELO CHELADA</t>
         </is>
       </c>
-      <c r="P15" s="2" t="inlineStr">
+      <c r="P23" s="2" t="inlineStr">
         <is>
           <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
-      <c r="Q15" s="3" t="inlineStr">
+      <c r="Q23" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
@@ -1794,6 +2470,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1838,7 +2522,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>09/11/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cooler doors from Promos_Report_15; "View photo" on the hub's Completed rows
Off-prem September: --merge-cooler-doors kept the report's 30 Cooler
Door Wrap rows (8 new); distinct stickers 20 -> 25 (Jayson Romine 0 -> 4,
Matthew Powierski 0 -> 1), still 2 reps at goal. The report carried no
new Bardstown menu row, so the on-prem archive is unchanged.

Hub: photo-verified objectives (cooler door stickers, Bardstown menu,
Lytt POS pics) now keep the tracker line's photo URL, and each Completed
row shows a "View photo" pill that opens the picture, mirroring the MPO
board's View Photo link. Cache tag bumped.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016mJ1rbpsvvg6uRmVytpP2z
</commit_message>
<xml_diff>
--- a/MPOs/off-prem/pos_cooler_door_promos.xlsx
+++ b/MPOs/off-prem/pos_cooler_door_promos.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q23"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.7109375" customWidth="1" style="6" min="1" max="1"/>
@@ -591,22 +591,22 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 10:37 AM</t>
+          <t>09/10/2026 11:46 AM</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Matthew Powierski</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -629,27 +629,27 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>WINELAND</t>
+          <t>WINE GRAND (CARLSTADT)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>50020</t>
+          <t>32017</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>247 DEGRAW AVE</t>
+          <t>675 PATERSON AVE</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>TEANECK</t>
+          <t>CARLSTADT</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -659,10 +659,14 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>MONACO</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="n"/>
+          <t>KEYSTONE ICE</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
+        </is>
+      </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -672,17 +676,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 12:28 PM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -706,31 +710,31 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK WINE/SPIRITS</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>88005</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>23 WYCKOFF AVE</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -740,12 +744,12 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>ATHLETIC BREWING CO</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>ATHLETIC BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q3" s="3" t="inlineStr">
@@ -757,17 +761,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 12:28 PM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -795,27 +799,27 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK WINE/SPIRITS</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>88005</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>23 WYCKOFF AVE</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>WALDWICK</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -825,12 +829,12 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>BLUE MOON BELGIAN WHITE ALE</t>
+          <t>TALKHOUSE ENCORE VARIETY PACK</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>TALKHOUSE ENCORE</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr">
@@ -842,22 +846,22 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 12:17 PM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Derrick laws</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -880,27 +884,27 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>RAPHAEL &amp; ANGEL LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>20080</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>390 MAIN ST</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -910,12 +914,12 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>SUN CRUISER ICED TEA + VODKA, CLASSIC ICED TEA</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q5" s="3" t="inlineStr">
@@ -927,22 +931,22 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:37 AM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>8.2</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Derrick laws</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -965,27 +969,27 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>THE LIQUOR SHOP</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>21033</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>498 E 30TH STREET</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -995,12 +999,12 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>MODELO CHELADA</t>
+          <t>SUN CRUISER ICED TEA + VODKA, HALF &amp; HALF</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q6" s="3" t="inlineStr">
@@ -1012,22 +1016,22 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:35 AM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>8.3</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Derrick laws</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1050,27 +1054,27 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>THE LIQUOR SHOP</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>21033</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>498 E 30TH STREET</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1080,12 +1084,12 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>CERVEZA REPUBLICA LA TUYA 5.0 LA DURA</t>
+          <t>SUN CRUISER ICED TEA VODKA VARIETY 18 PACK</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>VINAIO IMPORTS LTD</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q7" s="3" t="inlineStr">
@@ -1097,22 +1101,22 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:34 AM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>8.4</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Derrick laws</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1135,27 +1139,27 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>THE LIQUOR SHOP</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>21033</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>498 E 30TH STREET</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1165,12 +1169,12 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>MODELO ORO</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr">
@@ -1182,22 +1186,22 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>09/08/2026 11:32 AM</t>
+          <t>09/09/2026 12:40 PM</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>9.1</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Derrick laws</t>
+          <t>Jayson Romine</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Denise Montes</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1216,31 +1220,31 @@
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>THE LIQUOR SHOP</t>
+          <t>USA WINE TRADERS CLUB OF NEWTON (A)</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>21033</t>
+          <t>230412</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>498 E 30TH STREET</t>
+          <t>17 HAMPTON HOUSE ROAD</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>NEWTON</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>None</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1250,12 +1254,12 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>CAPE MAY BREWING COMPANY</t>
         </is>
       </c>
       <c r="Q9" s="3" t="inlineStr">
@@ -1267,7 +1271,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:34 AM</t>
+          <t>09/09/2026 10:37 AM</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1305,22 +1309,22 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>WINELAND</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>50020</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>247 DEGRAW AVE</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>TEANECK</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1335,14 +1339,10 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>CARBLISS</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>DRINK CARBLISS</t>
-        </is>
-      </c>
+          <t>MONACO</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="n"/>
       <c r="Q10" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
@@ -1352,7 +1352,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:33 AM</t>
+          <t>09/08/2026 12:28 PM</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1362,12 +1362,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1390,22 +1390,22 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -1420,7 +1420,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>TRULY HARD SELTZER</t>
+          <t>SUN CRUISERS RTD</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1437,7 +1437,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:32 AM</t>
+          <t>09/08/2026 12:28 PM</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1447,12 +1447,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Mike Ast</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Paul Deady</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1475,22 +1475,22 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>WALDWICK WINE/SPIRITS</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>88005</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>23 WYCKOFF AVE</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>WALDWICK</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>BLUE MOON BELGIAN WHITE ALE</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1522,7 +1522,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:31 AM</t>
+          <t>09/08/2026 12:17 PM</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1532,12 +1532,12 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -1560,22 +1560,22 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>RAPHAEL &amp; ANGEL LIQ (A)</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>20080</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>390 MAIN ST</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1590,12 +1590,12 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q13" s="3" t="inlineStr">
@@ -1607,22 +1607,22 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:31 AM</t>
+          <t>09/08/2026 11:37 AM</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1645,22 +1645,22 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -1675,7 +1675,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>MODELO CHELADA</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1692,22 +1692,22 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:30 AM</t>
+          <t>09/08/2026 11:35 AM</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1730,22 +1730,22 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -1760,12 +1760,12 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>CERVEZA REPUBLICA LA TUYA 5.0 LA DURA</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>CAPE MAY BREWING COMPANY</t>
+          <t>VINAIO IMPORTS LTD</t>
         </is>
       </c>
       <c r="Q15" s="3" t="inlineStr">
@@ -1777,22 +1777,22 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:29 AM</t>
+          <t>09/08/2026 11:34 AM</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1815,22 +1815,22 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -1845,12 +1845,12 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>MODELO ORO</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q16" s="3" t="inlineStr">
@@ -1862,22 +1862,22 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 11:11 AM</t>
+          <t>09/08/2026 11:32 AM</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>8.1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Mike Ast</t>
+          <t>Derrick laws</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
+          <t>Denise Montes</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -1900,22 +1900,22 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>FAIR LAWN WINE &amp; SPIRITS</t>
+          <t>THE LIQUOR SHOP</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>81006</t>
+          <t>21033</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>21-00 MAPLE AVE</t>
+          <t>498 E 30TH STREET</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>FAIR LAWN</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
@@ -1930,12 +1930,12 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>SUN CRUISERS RTD</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>BOSTON BEER COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q17" s="3" t="inlineStr">
@@ -1947,12 +1947,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:31 AM</t>
+          <t>09/03/2026 11:34 AM</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1985,22 +1985,22 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -2032,12 +2032,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:30 AM</t>
+          <t>09/03/2026 11:33 AM</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>9.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -2070,22 +2070,22 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -2100,12 +2100,12 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>CORONA EXTRA</t>
+          <t>TRULY HARD SELTZER</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>BOSTON BEER COMPANY</t>
         </is>
       </c>
       <c r="Q19" s="3" t="inlineStr">
@@ -2117,12 +2117,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:29 AM</t>
+          <t>09/03/2026 11:32 AM</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2155,22 +2155,22 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -2185,12 +2185,12 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>MODELO ESPECIAL</t>
+          <t>COORS LIGHT BEER</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>CONSTELLATION BRANDS</t>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
         </is>
       </c>
       <c r="Q20" s="3" t="inlineStr">
@@ -2202,12 +2202,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:28 AM</t>
+          <t>09/03/2026 11:31 AM</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2240,22 +2240,22 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -2270,12 +2270,12 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>COORS LIGHT BEER</t>
+          <t>CORONA EXTRA</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q21" s="3" t="inlineStr">
@@ -2287,12 +2287,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>09/03/2026 10:28 AM</t>
+          <t>09/03/2026 11:31 AM</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>11.2</t>
+          <t>4.2</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2325,22 +2325,22 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON DISC LIQ (A)</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>25045</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>73 ACKERMAN AVE BOTONY PL</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>CLIFTON</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -2355,12 +2355,12 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>MILLER LITE BEER</t>
+          <t>MODELO ESPECIAL</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>MOLSON COORS BEVERAGE COMPANY</t>
+          <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
       <c r="Q22" s="3" t="inlineStr">
@@ -2372,83 +2372,763 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>09/03/2026 11:30 AM</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>76010</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>66 MARKET ST</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>SADDLE BROOK</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>CAPE MAY BREWING COMPANY</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>CAPE MAY BREWING COMPANY</t>
+        </is>
+      </c>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 11:29 AM</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>6.1</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>76010</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>66 MARKET ST</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>SADDLE BROOK</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>SUN CRUISERS RTD</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>BOSTON BEER COMPANY</t>
+        </is>
+      </c>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 11:11 AM</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>7.1</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Mike Ast</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>FAIR LAWN WINE &amp; SPIRITS</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>81006</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>21-00 MAPLE AVE</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>FAIR LAWN</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>SUN CRUISERS RTD</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>BOSTON BEER COMPANY</t>
+        </is>
+      </c>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:31 AM</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>8.1</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>CARBLISS</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>DRINK CARBLISS</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:30 AM</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>9.1</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>CORONA EXTRA</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>CONSTELLATION BRANDS</t>
+        </is>
+      </c>
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:29 AM</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>MODELO ESPECIAL</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>CONSTELLATION BRANDS</t>
+        </is>
+      </c>
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:28 AM</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>11.1</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>COORS LIGHT BEER</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
+        </is>
+      </c>
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>09/03/2026 10:28 AM</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>11.2</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Chris Payton</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON DISC LIQ (A)</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>25045</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>73 ACKERMAN AVE BOTONY PL</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>CLIFTON</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>MBO</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>Cooler Door Wrap</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>MILLER LITE BEER</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>MOLSON COORS BEVERAGE COMPANY</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t>09/03/2026 10:27 AM</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>12.1</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Chris Payton</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Michael Engel</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Ashley Furman</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Sales Rep</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>Feature Activation</t>
         </is>
       </c>
-      <c r="H23" s="2" t="n">
+      <c r="H31" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>CLIFTON DISC LIQ (A)</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>25045</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>73 ACKERMAN AVE BOTONY PL</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>CLIFTON</t>
         </is>
       </c>
-      <c r="M23" s="2" t="inlineStr">
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>MBO</t>
         </is>
       </c>
-      <c r="N23" s="2" t="inlineStr">
+      <c r="N31" s="2" t="inlineStr">
         <is>
           <t>Cooler Door Wrap</t>
         </is>
       </c>
-      <c r="O23" s="2" t="inlineStr">
+      <c r="O31" s="2" t="inlineStr">
         <is>
           <t>MODELO CHELADA</t>
         </is>
       </c>
-      <c r="P23" s="2" t="inlineStr">
+      <c r="P31" s="2" t="inlineStr">
         <is>
           <t>CONSTELLATION BRANDS</t>
         </is>
       </c>
-      <c r="Q23" s="3" t="inlineStr">
+      <c r="Q31" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
@@ -2478,6 +3158,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>